<commit_message>
Add a logger and remove setup sheets
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -13,29 +13,25 @@
     <sheet name="Rooms" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="Speakers" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="Talks" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="talkTypeOfTimeslot_setup" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="talkTypeOfTimeslot_timeslotWithMatchingTalkType" sheetId="7" state="visible" r:id="rId8"/>
-    <sheet name="talkTypeOfTimeslot_timeslotWithNonMatchingTalkType" sheetId="8" state="visible" r:id="rId9"/>
-    <sheet name="talkHasUnavailableRoom_setup" sheetId="9" state="visible" r:id="rId10"/>
-    <sheet name="talkHasUnavailableRoom_talkWithAvailableRoom" sheetId="10" state="visible" r:id="rId11"/>
-    <sheet name="talkHasUnavailableRoom_talkWithUnavailableRoom" sheetId="11" state="visible" r:id="rId12"/>
-    <sheet name="talkHasUnavailableRoom_talkWithAvailableRoom_2" sheetId="12" state="visible" r:id="rId13"/>
-    <sheet name="talkHasUnavailableRoom_talkWithUnavailableRoom_2" sheetId="13" state="visible" r:id="rId14"/>
-    <sheet name="roomConflict_setup" sheetId="14" state="visible" r:id="rId15"/>
-    <sheet name="roomConflict_talksInSameRoomWithoutOverlappingTimeslots" sheetId="15" state="visible" r:id="rId16"/>
-    <sheet name="roomConflict_talksInSameRoomWithOverlappingTimeslots" sheetId="16" state="visible" r:id="rId17"/>
-    <sheet name="roomConflict_talksInDifferentRoomsWithOverlappingTimeslots" sheetId="17" state="visible" r:id="rId18"/>
-    <sheet name="talkWithUnavailableSpeaker_setup" sheetId="18" state="visible" r:id="rId19"/>
-    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableSpeaker" sheetId="19" state="visible" r:id="rId20"/>
-    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableSpeaker_2" sheetId="20" state="visible" r:id="rId21"/>
-    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableTwoSpeakers" sheetId="21" state="visible" r:id="rId22"/>
-    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableTwoSpeakers_2" sheetId="22" state="visible" r:id="rId23"/>
-    <sheet name="talkWithUnavailableSpeaker_talkWithOneOrMoreUnavailableSpeaker" sheetId="23" state="visible" r:id="rId24"/>
-    <sheet name="talkWithUnavailableSpeaker_talkWithOneOrMoreUnavailableSpeaker_2" sheetId="24" state="visible" r:id="rId25"/>
-    <sheet name="talkWithUnavailableSpeaker_talkWithOneOrMoreUnavailableSpeaker_3" sheetId="25" state="visible" r:id="rId26"/>
-    <sheet name="speakerConflict_setup" sheetId="26" state="visible" r:id="rId27"/>
-    <sheet name="speakerConflict_speakerHasNoConflictingTimeslots" sheetId="27" state="visible" r:id="rId28"/>
-    <sheet name="speakerConflict_speakerHasConflictingTimeslots" sheetId="28" state="visible" r:id="rId29"/>
+    <sheet name="talkTypeOfTimeslot_timeslotWithMatchingTalkType" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="talkTypeOfTimeslot_timeslotWithNonMatchingTalkType" sheetId="7" state="visible" r:id="rId8"/>
+    <sheet name="talkHasUnavailableRoom_setup" sheetId="8" state="visible" r:id="rId9"/>
+    <sheet name="talkHasUnavailableRoom_talkWithAvailableRoom" sheetId="9" state="visible" r:id="rId10"/>
+    <sheet name="talkHasUnavailableRoom_talkWithUnavailableRoom" sheetId="10" state="visible" r:id="rId11"/>
+    <sheet name="talkHasUnavailableRoom_talkWithAvailableRoom_2" sheetId="11" state="visible" r:id="rId12"/>
+    <sheet name="talkHasUnavailableRoom_talkWithUnavailableRoom_2" sheetId="12" state="visible" r:id="rId13"/>
+    <sheet name="roomConflict_talksInSameRoomWithoutOverlappingTimeslots" sheetId="13" state="visible" r:id="rId14"/>
+    <sheet name="roomConflict_talksInSameRoomWithOverlappingTimeslots" sheetId="14" state="visible" r:id="rId15"/>
+    <sheet name="roomConflict_talksInDifferentRoomsWithOverlappingTimeslots" sheetId="15" state="visible" r:id="rId16"/>
+    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableSpeaker" sheetId="16" state="visible" r:id="rId17"/>
+    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableSpeaker_2" sheetId="17" state="visible" r:id="rId18"/>
+    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableTwoSpeakers" sheetId="18" state="visible" r:id="rId19"/>
+    <sheet name="talkWithUnavailableSpeaker_talkWithoutUnavailableTwoSpeakers_2" sheetId="19" state="visible" r:id="rId20"/>
+    <sheet name="talkWithUnavailableSpeaker_talkWithOneOrMoreUnavailableSpeaker" sheetId="20" state="visible" r:id="rId21"/>
+    <sheet name="talkWithUnavailableSpeaker_talkWithOneOrMoreUnavailableSpeaker_2" sheetId="21" state="visible" r:id="rId22"/>
+    <sheet name="talkWithUnavailableSpeaker_talkWithOneOrMoreUnavailableSpeaker_3" sheetId="22" state="visible" r:id="rId23"/>
+    <sheet name="speakerConflict_speakerHasNoConflictingTimeslots" sheetId="23" state="visible" r:id="rId24"/>
+    <sheet name="speakerConflict_speakerHasConflictingTimeslots" sheetId="24" state="visible" r:id="rId25"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -47,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="140">
   <si>
     <t xml:space="preserve">Conference name</t>
   </si>
@@ -1257,7 +1253,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1327,9 +1323,6 @@
       <c r="A7" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="C7" s="6"/>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
@@ -1346,7 +1339,6 @@
       <c r="A8" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="6"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
@@ -1363,7 +1355,9 @@
       <c r="A9" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="C9" s="11"/>
       <c r="D9" s="4"/>
       <c r="E9" s="11"/>
@@ -1470,7 +1464,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1556,6 +1550,9 @@
       <c r="A8" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B8" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
@@ -1572,9 +1569,7 @@
       <c r="A9" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>117</v>
-      </c>
+      <c r="B9" s="4"/>
       <c r="C9" s="11"/>
       <c r="D9" s="4"/>
       <c r="E9" s="11"/>
@@ -1681,7 +1676,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1767,9 +1762,6 @@
       <c r="A8" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
@@ -1786,7 +1778,6 @@
       <c r="A9" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="4"/>
       <c r="C9" s="11"/>
       <c r="D9" s="4"/>
       <c r="E9" s="11"/>
@@ -1803,7 +1794,9 @@
       <c r="A10" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B10" s="1"/>
+      <c r="B10" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -1843,7 +1836,7 @@
     <tabColor rgb="FF00DCFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
@@ -1875,7 +1868,7 @@
         <v>133</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1893,7 +1886,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1924,10 +1917,10 @@
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="11"/>
+      <c r="D5" s="4"/>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
@@ -1945,10 +1938,12 @@
       <c r="B6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="D6" s="12"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -1960,11 +1955,16 @@
       <c r="M6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>81</v>
+      <c r="A7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>119</v>
       </c>
       <c r="C7" s="6"/>
-      <c r="D7" s="7"/>
+      <c r="D7" s="7" t="s">
+        <v>120</v>
+      </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -1976,9 +1976,10 @@
       <c r="M7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>82</v>
-      </c>
+      <c r="A8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="6"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
@@ -1991,41 +1992,8 @@
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
     </row>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-    </row>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2033,9 +2001,8 @@
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="F9:H9"/>
+  <mergeCells count="1">
+    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2103,7 +2070,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -2175,9 +2142,12 @@
       <c r="A7" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="7"/>
+      <c r="B7" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>120</v>
+      </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -2355,12 +2325,8 @@
       <c r="A7" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="7" t="s">
-        <v>120</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -2377,7 +2343,9 @@
         <v>86</v>
       </c>
       <c r="B8" s="6"/>
-      <c r="C8" s="7"/>
+      <c r="C8" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
       <c r="F8" s="7"/>
@@ -2417,7 +2385,7 @@
     <tabColor rgb="FF00DCFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
@@ -2448,8 +2416,8 @@
       <c r="A2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>38</v>
+      <c r="B2" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -2467,7 +2435,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -2498,10 +2466,10 @@
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="11"/>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
@@ -2519,12 +2487,10 @@
       <c r="B6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" s="12" t="s">
+      <c r="C6" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="D6" s="12"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -2537,14 +2503,13 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>120</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -2555,23 +2520,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2582,7 +2531,7 @@
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B5:C5"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2600,7 +2549,7 @@
     <tabColor rgb="FF00DCFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
@@ -2631,8 +2580,8 @@
       <c r="A2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>38</v>
+      <c r="B2" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -2681,10 +2630,10 @@
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="11"/>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
@@ -2702,12 +2651,10 @@
       <c r="B6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" s="12" t="s">
+      <c r="C6" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="D6" s="12"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -2720,11 +2667,12 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>119</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="7"/>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -2735,25 +2683,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2764,7 +2694,7 @@
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B5:C5"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2902,8 +2832,9 @@
       <c r="A7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
+      <c r="B7" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -3064,10 +2995,10 @@
       <c r="A7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C7" s="6"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -3412,7 +3343,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -3482,8 +3413,8 @@
       <c r="A7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>121</v>
+      <c r="B7" s="2" t="s">
+        <v>124</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
@@ -3575,7 +3506,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -3646,7 +3577,7 @@
         <v>87</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
@@ -3738,7 +3669,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -3808,9 +3739,8 @@
       <c r="A7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2" t="s">
-        <v>122</v>
+      <c r="B7" s="2" t="s">
+        <v>127</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
@@ -3884,7 +3814,7 @@
         <v>133</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -3902,7 +3832,7 @@
         <v>134</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -3933,495 +3863,6 @@
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-    </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B5:C5"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="false">
-    <tabColor rgb="FF00DCFF"/>
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="0" width="19.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="0" width="8.67"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-    </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B5:C5"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="false">
-    <tabColor rgb="FF00DCFF"/>
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="0" width="19.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="0" width="8.67"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-    </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B5:C5"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="false">
-    <tabColor rgb="FF00DCFF"/>
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="0" width="19.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="0" width="8.67"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C5" s="4"/>
@@ -4463,9 +3904,13 @@
       <c r="A7" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="C7" s="6"/>
-      <c r="D7" s="7"/>
+      <c r="D7" s="3" t="s">
+        <v>130</v>
+      </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -4499,175 +3944,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="false">
-    <tabColor rgb="FF00DCFF"/>
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="0" width="19.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="0" width="8.67"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-    </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B5:D5"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <tabColor rgb="FF00DCFF"/>
@@ -7735,7 +7012,9 @@
       <c r="A7" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="13" t="s">
+        <v>115</v>
+      </c>
       <c r="C7" s="6"/>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
@@ -7900,7 +7179,9 @@
       <c r="B7" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="6"/>
+      <c r="C7" s="13" t="s">
+        <v>116</v>
+      </c>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -7941,7 +7222,7 @@
     <tabColor rgb="FF00DCFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
@@ -7972,8 +7253,8 @@
       <c r="A2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>33</v>
+      <c r="B2" s="14" t="s">
+        <v>36</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -8022,7 +7303,7 @@
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="11"/>
@@ -8059,14 +7340,10 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>116</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -8078,9 +7355,57 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+    </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8088,8 +7413,9 @@
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F9:H9"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -8227,7 +7553,9 @@
       <c r="A7" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="C7" s="6"/>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>

</xml_diff>

<commit_message>
Remove unnecessary fields and fix indentations
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="117">
   <si>
     <t xml:space="preserve">Conference name</t>
   </si>
@@ -265,9 +265,6 @@
   </si>
   <si>
     <t xml:space="preserve">unavailableRoom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fri 2018-01-05</t>
   </si>
   <si>
     <t xml:space="preserve">Required timeslot tags</t>
@@ -518,11 +515,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1014,10 +1011,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1032,7 +1029,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>38</v>
@@ -1050,10 +1047,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1100,7 +1097,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -1125,20 +1122,20 @@
       <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -1182,10 +1179,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1200,7 +1197,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>38</v>
@@ -1218,10 +1215,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1268,7 +1265,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -1293,19 +1290,19 @@
       <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -1349,10 +1346,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1367,7 +1364,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>38</v>
@@ -1385,10 +1382,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1435,7 +1432,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -1461,15 +1458,15 @@
         <v>73</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="4"/>
+        <v>101</v>
+      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -1477,18 +1474,18 @@
       <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D8" s="8"/>
-      <c r="E8" s="4"/>
+      <c r="E8" s="5"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
-      <c r="H8" s="4"/>
+      <c r="H8" s="5"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
-      <c r="K8" s="4"/>
+      <c r="K8" s="5"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
     </row>
@@ -1531,10 +1528,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1549,7 +1546,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>40</v>
@@ -1567,10 +1564,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1617,7 +1614,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -1643,16 +1640,16 @@
         <v>73</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -1696,10 +1693,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1714,7 +1711,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>40</v>
@@ -1732,10 +1729,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1782,7 +1779,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -1809,16 +1806,16 @@
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -1862,10 +1859,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1880,7 +1877,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>40</v>
@@ -1898,10 +1895,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1948,7 +1945,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -1974,16 +1971,16 @@
         <v>73</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -2027,10 +2024,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -2043,9 +2040,9 @@
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>40</v>
@@ -2063,10 +2060,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -2113,7 +2110,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -2139,16 +2136,16 @@
         <v>73</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -2192,10 +2189,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -2210,7 +2207,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>42</v>
@@ -2228,10 +2225,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -2278,7 +2275,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -2304,19 +2301,19 @@
         <v>73</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="4"/>
+        <v>101</v>
+      </c>
+      <c r="C7" s="5"/>
       <c r="D7" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E7" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -2360,10 +2357,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -2378,7 +2375,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>42</v>
@@ -2396,10 +2393,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -2446,7 +2443,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -2472,15 +2469,15 @@
         <v>73</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="4"/>
+        <v>101</v>
+      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -2488,18 +2485,18 @@
       <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D8" s="8"/>
-      <c r="E8" s="4"/>
+      <c r="E8" s="5"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
-      <c r="H8" s="4"/>
+      <c r="H8" s="5"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
-      <c r="K8" s="4"/>
+      <c r="K8" s="5"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
     </row>
@@ -2634,7 +2631,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.49"/>
@@ -2700,25 +2697,17 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+    <row r="5" customFormat="false" ht="35.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2771,9 +2760,7 @@
       </c>
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
-      <c r="M1" s="3" t="s">
-        <v>76</v>
-      </c>
+      <c r="M1" s="3"/>
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
     </row>
@@ -2782,28 +2769,28 @@
         <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>70</v>
@@ -2814,19 +2801,13 @@
       <c r="L2" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>72</v>
-      </c>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -2837,15 +2818,15 @@
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -2856,15 +2837,15 @@
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
       <c r="M4" s="8"/>
       <c r="N4" s="8"/>
       <c r="O4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -2875,15 +2856,15 @@
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="6"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
       <c r="O5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -2950,64 +2931,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>57</v>
@@ -3016,19 +2997,19 @@
         <v>58</v>
       </c>
       <c r="W1" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>102</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -3054,14 +3035,14 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -3085,15 +3066,23 @@
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="C4" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>105</v>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -3110,16 +3099,16 @@
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -3143,16 +3132,16 @@
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -3200,39 +3189,6 @@
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2"/>
@@ -4706,10 +4662,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -4724,7 +4680,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>33</v>
@@ -4742,10 +4698,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -4792,7 +4748,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -4818,17 +4774,17 @@
         <v>73</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="4"/>
+        <v>101</v>
+      </c>
+      <c r="C7" s="5"/>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -4872,10 +4828,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -4890,7 +4846,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>33</v>
@@ -4908,10 +4864,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -4958,7 +4914,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -4980,21 +4936,21 @@
       <c r="M6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -5038,10 +4994,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -5056,7 +5012,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>36</v>
@@ -5074,10 +5030,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -5124,7 +5080,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -5146,21 +5102,21 @@
       <c r="M6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="4"/>
+      <c r="B7" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="5"/>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
@@ -5204,10 +5160,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -5222,7 +5178,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>36</v>
@@ -5240,10 +5196,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -5290,7 +5246,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -5312,20 +5268,20 @@
       <c r="M6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>102</v>
+      <c r="C7" s="5" t="s">
+        <v>101</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="5"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="4"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>

</xml_diff>

<commit_message>
Convert into parameterized test
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -398,7 +398,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -428,20 +428,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="4">
@@ -498,7 +488,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -515,23 +505,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -543,19 +521,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1013,14 +983,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1031,14 +1001,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="8" t="s">
         <v>38</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1049,14 +1019,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -1065,13 +1035,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -1085,15 +1055,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -1102,42 +1072,42 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1181,14 +1151,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1199,14 +1169,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="8" t="s">
         <v>38</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1217,14 +1187,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>115</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -1233,13 +1203,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -1253,15 +1223,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -1270,41 +1240,41 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1348,14 +1318,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1366,14 +1336,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="8" t="s">
         <v>38</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1384,14 +1354,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -1400,13 +1370,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -1420,15 +1390,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -1437,21 +1407,21 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -1460,34 +1430,34 @@
       <c r="B7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="5"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1530,14 +1500,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1548,14 +1518,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>40</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1566,14 +1536,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -1582,13 +1552,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -1602,15 +1572,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -1619,21 +1589,21 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -1642,16 +1612,16 @@
       <c r="C7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1695,14 +1665,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1713,14 +1683,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>40</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1731,14 +1701,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -1747,13 +1717,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -1767,15 +1737,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -1784,21 +1754,21 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -1808,16 +1778,16 @@
       <c r="C7" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1861,14 +1831,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1879,14 +1849,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>40</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1897,14 +1867,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>116</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -1913,13 +1883,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -1933,15 +1903,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -1950,21 +1920,21 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -1973,16 +1943,16 @@
       <c r="B7" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2026,14 +1996,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -2044,14 +2014,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>40</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -2062,14 +2032,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>116</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -2078,13 +2048,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -2098,15 +2068,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -2115,21 +2085,21 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -2138,16 +2108,16 @@
       <c r="B7" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2191,14 +2161,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -2209,14 +2179,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -2227,14 +2197,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -2243,13 +2213,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -2263,15 +2233,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -2286,15 +2256,15 @@
       <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -2303,19 +2273,19 @@
       <c r="B7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="5"/>
+      <c r="C7" s="4"/>
       <c r="D7" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2359,14 +2329,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -2377,14 +2347,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -2395,14 +2365,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>116</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -2411,13 +2381,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -2431,15 +2401,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -2454,15 +2424,15 @@
       <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -2471,34 +2441,34 @@
       <c r="B7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="5"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2698,16 +2668,16 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="35.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="5"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2795,10 +2765,10 @@
       <c r="J2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="1" t="s">
         <v>72</v>
       </c>
       <c r="M2" s="1"/>
@@ -2809,77 +2779,77 @@
       <c r="A3" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3001,7 +2971,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>101</v>
       </c>
       <c r="B2" s="2"/>
@@ -3027,7 +2997,7 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
-      <c r="S2" s="9"/>
+      <c r="S2" s="6"/>
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
@@ -3060,7 +3030,7 @@
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
-      <c r="S3" s="9"/>
+      <c r="S3" s="6"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
@@ -3093,7 +3063,7 @@
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
-      <c r="S4" s="9"/>
+      <c r="S4" s="6"/>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
@@ -3126,7 +3096,7 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
-      <c r="S5" s="9"/>
+      <c r="S5" s="6"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
@@ -3159,7 +3129,7 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
-      <c r="S6" s="9"/>
+      <c r="S6" s="6"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
@@ -3184,7 +3154,7 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
-      <c r="S7" s="9"/>
+      <c r="S7" s="6"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
@@ -3209,7 +3179,7 @@
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
-      <c r="S9" s="9"/>
+      <c r="S9" s="6"/>
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
@@ -3234,7 +3204,7 @@
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
-      <c r="S10" s="9"/>
+      <c r="S10" s="6"/>
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
@@ -3259,7 +3229,7 @@
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
-      <c r="S11" s="9"/>
+      <c r="S11" s="6"/>
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
@@ -3284,7 +3254,7 @@
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
-      <c r="S12" s="9"/>
+      <c r="S12" s="6"/>
       <c r="T12" s="2"/>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
@@ -3309,7 +3279,7 @@
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
-      <c r="S13" s="9"/>
+      <c r="S13" s="6"/>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
@@ -3334,7 +3304,7 @@
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
-      <c r="S14" s="9"/>
+      <c r="S14" s="6"/>
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
@@ -3359,7 +3329,7 @@
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
-      <c r="S15" s="9"/>
+      <c r="S15" s="6"/>
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
@@ -3384,7 +3354,7 @@
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
-      <c r="S16" s="9"/>
+      <c r="S16" s="6"/>
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
@@ -3409,7 +3379,7 @@
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
-      <c r="S17" s="9"/>
+      <c r="S17" s="6"/>
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
@@ -3434,7 +3404,7 @@
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
-      <c r="S18" s="9"/>
+      <c r="S18" s="6"/>
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
@@ -3459,7 +3429,7 @@
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
-      <c r="S19" s="9"/>
+      <c r="S19" s="6"/>
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
@@ -3484,7 +3454,7 @@
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
-      <c r="S20" s="9"/>
+      <c r="S20" s="6"/>
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
@@ -3509,7 +3479,7 @@
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
-      <c r="S21" s="9"/>
+      <c r="S21" s="6"/>
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
@@ -3534,7 +3504,7 @@
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
-      <c r="S22" s="9"/>
+      <c r="S22" s="6"/>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
@@ -3559,7 +3529,7 @@
       <c r="P23" s="2"/>
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
-      <c r="S23" s="9"/>
+      <c r="S23" s="6"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
@@ -3584,7 +3554,7 @@
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
-      <c r="S24" s="9"/>
+      <c r="S24" s="6"/>
       <c r="T24" s="2"/>
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
@@ -3609,7 +3579,7 @@
       <c r="P25" s="2"/>
       <c r="Q25" s="2"/>
       <c r="R25" s="2"/>
-      <c r="S25" s="9"/>
+      <c r="S25" s="6"/>
       <c r="T25" s="2"/>
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
@@ -3634,7 +3604,7 @@
       <c r="P26" s="2"/>
       <c r="Q26" s="2"/>
       <c r="R26" s="2"/>
-      <c r="S26" s="9"/>
+      <c r="S26" s="6"/>
       <c r="T26" s="2"/>
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
@@ -3659,7 +3629,7 @@
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
-      <c r="S27" s="9"/>
+      <c r="S27" s="6"/>
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
@@ -3684,7 +3654,7 @@
       <c r="P28" s="2"/>
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
-      <c r="S28" s="9"/>
+      <c r="S28" s="6"/>
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
@@ -3709,7 +3679,7 @@
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
-      <c r="S29" s="9"/>
+      <c r="S29" s="6"/>
       <c r="T29" s="2"/>
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
@@ -3734,7 +3704,7 @@
       <c r="P30" s="2"/>
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
-      <c r="S30" s="9"/>
+      <c r="S30" s="6"/>
       <c r="T30" s="2"/>
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
@@ -3759,7 +3729,7 @@
       <c r="P31" s="2"/>
       <c r="Q31" s="2"/>
       <c r="R31" s="2"/>
-      <c r="S31" s="9"/>
+      <c r="S31" s="6"/>
       <c r="T31" s="2"/>
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
@@ -3784,7 +3754,7 @@
       <c r="P32" s="2"/>
       <c r="Q32" s="2"/>
       <c r="R32" s="2"/>
-      <c r="S32" s="9"/>
+      <c r="S32" s="6"/>
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
@@ -3809,7 +3779,7 @@
       <c r="P33" s="2"/>
       <c r="Q33" s="2"/>
       <c r="R33" s="2"/>
-      <c r="S33" s="9"/>
+      <c r="S33" s="6"/>
       <c r="T33" s="2"/>
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
@@ -3834,7 +3804,7 @@
       <c r="P34" s="2"/>
       <c r="Q34" s="2"/>
       <c r="R34" s="2"/>
-      <c r="S34" s="9"/>
+      <c r="S34" s="6"/>
       <c r="T34" s="2"/>
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
@@ -3859,7 +3829,7 @@
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
       <c r="R35" s="2"/>
-      <c r="S35" s="9"/>
+      <c r="S35" s="6"/>
       <c r="T35" s="2"/>
       <c r="U35" s="2"/>
       <c r="V35" s="2"/>
@@ -3884,7 +3854,7 @@
       <c r="P36" s="2"/>
       <c r="Q36" s="2"/>
       <c r="R36" s="2"/>
-      <c r="S36" s="9"/>
+      <c r="S36" s="6"/>
       <c r="T36" s="2"/>
       <c r="U36" s="2"/>
       <c r="V36" s="2"/>
@@ -3909,7 +3879,7 @@
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
       <c r="R37" s="2"/>
-      <c r="S37" s="9"/>
+      <c r="S37" s="6"/>
       <c r="T37" s="2"/>
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
@@ -3934,7 +3904,7 @@
       <c r="P38" s="2"/>
       <c r="Q38" s="2"/>
       <c r="R38" s="2"/>
-      <c r="S38" s="9"/>
+      <c r="S38" s="6"/>
       <c r="T38" s="2"/>
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
@@ -3959,7 +3929,7 @@
       <c r="P39" s="2"/>
       <c r="Q39" s="2"/>
       <c r="R39" s="2"/>
-      <c r="S39" s="9"/>
+      <c r="S39" s="6"/>
       <c r="T39" s="2"/>
       <c r="U39" s="2"/>
       <c r="V39" s="2"/>
@@ -3984,7 +3954,7 @@
       <c r="P40" s="2"/>
       <c r="Q40" s="2"/>
       <c r="R40" s="2"/>
-      <c r="S40" s="9"/>
+      <c r="S40" s="6"/>
       <c r="T40" s="2"/>
       <c r="U40" s="2"/>
       <c r="V40" s="2"/>
@@ -4009,7 +3979,7 @@
       <c r="P41" s="2"/>
       <c r="Q41" s="2"/>
       <c r="R41" s="2"/>
-      <c r="S41" s="9"/>
+      <c r="S41" s="6"/>
       <c r="T41" s="2"/>
       <c r="U41" s="2"/>
       <c r="V41" s="2"/>
@@ -4034,7 +4004,7 @@
       <c r="P42" s="2"/>
       <c r="Q42" s="2"/>
       <c r="R42" s="2"/>
-      <c r="S42" s="9"/>
+      <c r="S42" s="6"/>
       <c r="T42" s="2"/>
       <c r="U42" s="2"/>
       <c r="V42" s="2"/>
@@ -4059,7 +4029,7 @@
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
-      <c r="S43" s="9"/>
+      <c r="S43" s="6"/>
       <c r="T43" s="2"/>
       <c r="U43" s="2"/>
       <c r="V43" s="2"/>
@@ -4084,7 +4054,7 @@
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
-      <c r="S44" s="9"/>
+      <c r="S44" s="6"/>
       <c r="T44" s="2"/>
       <c r="U44" s="2"/>
       <c r="V44" s="2"/>
@@ -4109,7 +4079,7 @@
       <c r="P45" s="2"/>
       <c r="Q45" s="2"/>
       <c r="R45" s="2"/>
-      <c r="S45" s="9"/>
+      <c r="S45" s="6"/>
       <c r="T45" s="2"/>
       <c r="U45" s="2"/>
       <c r="V45" s="2"/>
@@ -4134,7 +4104,7 @@
       <c r="P46" s="2"/>
       <c r="Q46" s="2"/>
       <c r="R46" s="2"/>
-      <c r="S46" s="9"/>
+      <c r="S46" s="6"/>
       <c r="T46" s="2"/>
       <c r="U46" s="2"/>
       <c r="V46" s="2"/>
@@ -4159,7 +4129,7 @@
       <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
       <c r="R47" s="2"/>
-      <c r="S47" s="9"/>
+      <c r="S47" s="6"/>
       <c r="T47" s="2"/>
       <c r="U47" s="2"/>
       <c r="V47" s="2"/>
@@ -4184,7 +4154,7 @@
       <c r="P48" s="2"/>
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
-      <c r="S48" s="9"/>
+      <c r="S48" s="6"/>
       <c r="T48" s="2"/>
       <c r="U48" s="2"/>
       <c r="V48" s="2"/>
@@ -4209,7 +4179,7 @@
       <c r="P49" s="2"/>
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
-      <c r="S49" s="9"/>
+      <c r="S49" s="6"/>
       <c r="T49" s="2"/>
       <c r="U49" s="2"/>
       <c r="V49" s="2"/>
@@ -4234,7 +4204,7 @@
       <c r="P50" s="2"/>
       <c r="Q50" s="2"/>
       <c r="R50" s="2"/>
-      <c r="S50" s="9"/>
+      <c r="S50" s="6"/>
       <c r="T50" s="2"/>
       <c r="U50" s="2"/>
       <c r="V50" s="2"/>
@@ -4259,7 +4229,7 @@
       <c r="P51" s="2"/>
       <c r="Q51" s="2"/>
       <c r="R51" s="2"/>
-      <c r="S51" s="9"/>
+      <c r="S51" s="6"/>
       <c r="T51" s="2"/>
       <c r="U51" s="2"/>
       <c r="V51" s="2"/>
@@ -4284,7 +4254,7 @@
       <c r="P52" s="2"/>
       <c r="Q52" s="2"/>
       <c r="R52" s="2"/>
-      <c r="S52" s="9"/>
+      <c r="S52" s="6"/>
       <c r="T52" s="2"/>
       <c r="U52" s="2"/>
       <c r="V52" s="2"/>
@@ -4309,7 +4279,7 @@
       <c r="P53" s="2"/>
       <c r="Q53" s="2"/>
       <c r="R53" s="2"/>
-      <c r="S53" s="9"/>
+      <c r="S53" s="6"/>
       <c r="T53" s="2"/>
       <c r="U53" s="2"/>
       <c r="V53" s="2"/>
@@ -4334,7 +4304,7 @@
       <c r="P54" s="2"/>
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
-      <c r="S54" s="9"/>
+      <c r="S54" s="6"/>
       <c r="T54" s="2"/>
       <c r="U54" s="2"/>
       <c r="V54" s="2"/>
@@ -4359,7 +4329,7 @@
       <c r="P55" s="2"/>
       <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
-      <c r="S55" s="9"/>
+      <c r="S55" s="6"/>
       <c r="T55" s="2"/>
       <c r="U55" s="2"/>
       <c r="V55" s="2"/>
@@ -4384,7 +4354,7 @@
       <c r="P56" s="2"/>
       <c r="Q56" s="2"/>
       <c r="R56" s="2"/>
-      <c r="S56" s="9"/>
+      <c r="S56" s="6"/>
       <c r="T56" s="2"/>
       <c r="U56" s="2"/>
       <c r="V56" s="2"/>
@@ -4409,7 +4379,7 @@
       <c r="P57" s="2"/>
       <c r="Q57" s="2"/>
       <c r="R57" s="2"/>
-      <c r="S57" s="9"/>
+      <c r="S57" s="6"/>
       <c r="T57" s="2"/>
       <c r="U57" s="2"/>
       <c r="V57" s="2"/>
@@ -4434,7 +4404,7 @@
       <c r="P58" s="2"/>
       <c r="Q58" s="2"/>
       <c r="R58" s="2"/>
-      <c r="S58" s="9"/>
+      <c r="S58" s="6"/>
       <c r="T58" s="2"/>
       <c r="U58" s="2"/>
       <c r="V58" s="2"/>
@@ -4459,7 +4429,7 @@
       <c r="P59" s="2"/>
       <c r="Q59" s="2"/>
       <c r="R59" s="2"/>
-      <c r="S59" s="9"/>
+      <c r="S59" s="6"/>
       <c r="T59" s="2"/>
       <c r="U59" s="2"/>
       <c r="V59" s="2"/>
@@ -4484,7 +4454,7 @@
       <c r="P60" s="2"/>
       <c r="Q60" s="2"/>
       <c r="R60" s="2"/>
-      <c r="S60" s="9"/>
+      <c r="S60" s="6"/>
       <c r="T60" s="2"/>
       <c r="U60" s="2"/>
       <c r="V60" s="2"/>
@@ -4509,7 +4479,7 @@
       <c r="P61" s="2"/>
       <c r="Q61" s="2"/>
       <c r="R61" s="2"/>
-      <c r="S61" s="9"/>
+      <c r="S61" s="6"/>
       <c r="T61" s="2"/>
       <c r="U61" s="2"/>
       <c r="V61" s="2"/>
@@ -4534,7 +4504,7 @@
       <c r="P62" s="2"/>
       <c r="Q62" s="2"/>
       <c r="R62" s="2"/>
-      <c r="S62" s="9"/>
+      <c r="S62" s="6"/>
       <c r="T62" s="2"/>
       <c r="U62" s="2"/>
       <c r="V62" s="2"/>
@@ -4559,7 +4529,7 @@
       <c r="P63" s="2"/>
       <c r="Q63" s="2"/>
       <c r="R63" s="2"/>
-      <c r="S63" s="9"/>
+      <c r="S63" s="6"/>
       <c r="T63" s="2"/>
       <c r="U63" s="2"/>
       <c r="V63" s="2"/>
@@ -4584,7 +4554,7 @@
       <c r="P64" s="2"/>
       <c r="Q64" s="2"/>
       <c r="R64" s="2"/>
-      <c r="S64" s="9"/>
+      <c r="S64" s="6"/>
       <c r="T64" s="2"/>
       <c r="U64" s="2"/>
       <c r="V64" s="2"/>
@@ -4609,7 +4579,7 @@
       <c r="P65" s="2"/>
       <c r="Q65" s="2"/>
       <c r="R65" s="2"/>
-      <c r="S65" s="10"/>
+      <c r="S65" s="7"/>
       <c r="T65" s="2"/>
       <c r="U65" s="2"/>
       <c r="V65" s="2"/>
@@ -4664,14 +4634,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -4682,14 +4652,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>33</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -4700,14 +4670,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -4716,13 +4686,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -4736,15 +4706,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -4753,21 +4723,21 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -4776,17 +4746,17 @@
       <c r="B7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4830,14 +4800,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -4848,14 +4818,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
         <v>33</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -4866,14 +4836,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -4882,13 +4852,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -4902,15 +4872,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -4919,40 +4889,40 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="13"/>
+      <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4996,14 +4966,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -5014,14 +4984,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="8" t="s">
         <v>36</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -5032,14 +5002,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -5048,13 +5018,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -5068,15 +5038,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -5085,40 +5055,40 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5162,14 +5132,14 @@
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="12"/>
+      <c r="H1" s="9"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -5180,14 +5150,14 @@
       <c r="A2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="8" t="s">
         <v>36</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12"/>
+      <c r="H2" s="9"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -5198,14 +5168,14 @@
       <c r="A3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12"/>
+      <c r="H3" s="9"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -5214,13 +5184,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12"/>
+      <c r="H4" s="9"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -5234,15 +5204,15 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -5251,39 +5221,39 @@
       <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Add testSheetName as the name of unit test
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Rooms" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="Speakers" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="Talks" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="talkTypeOfTimeslot_timeslotWithMatchingTalkType" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="talkTypeOfTimeslot_timeslotWithNonMatchingTalkType" sheetId="7" state="visible" r:id="rId8"/>
+    <sheet name="Talk type of timeslot 1" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="Talk type of timeslot 2" sheetId="7" state="visible" r:id="rId8"/>
     <sheet name="talkHasUnavailableRoom_talkWithAvailableRoom" sheetId="8" state="visible" r:id="rId9"/>
     <sheet name="talkHasUnavailableRoom_talkWithUnavailableRoom" sheetId="9" state="visible" r:id="rId10"/>
     <sheet name="roomConflict_talksInSameRoomWithoutOverlappingTimeslots" sheetId="10" state="visible" r:id="rId11"/>
@@ -4621,7 +4621,7 @@
     <tabColor rgb="FF00DCFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M1048576"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
@@ -4767,6 +4767,7 @@
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B5:D5"/>

</xml_diff>

<commit_message>
Set soft constraints' weights to 1
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="16"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -715,7 +715,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
@@ -726,7 +726,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -748,7 +748,7 @@
         <v>11</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
@@ -770,7 +770,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>16</v>
@@ -781,7 +781,7 @@
         <v>17</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>18</v>
@@ -792,7 +792,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>20</v>
@@ -803,7 +803,7 @@
         <v>21</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>22</v>
@@ -814,7 +814,7 @@
         <v>23</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>24</v>
@@ -825,7 +825,7 @@
         <v>25</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>22</v>
@@ -836,7 +836,7 @@
         <v>26</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>24</v>
@@ -847,7 +847,7 @@
         <v>27</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>28</v>
@@ -858,7 +858,7 @@
         <v>29</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>30</v>
@@ -869,7 +869,7 @@
         <v>31</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>28</v>
@@ -880,7 +880,7 @@
         <v>32</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Fix conference name in test file
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -42,7 +42,7 @@
     <t xml:space="preserve">Conference name</t>
   </si>
   <si>
-    <t xml:space="preserve">JayFocus 2023</t>
+    <t xml:space="preserve">Junit test</t>
   </si>
   <si>
     <t xml:space="preserve">Constraint</t>
@@ -691,7 +691,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="4" style="0" width="8.67"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add test cases for Talk prerequisite talks constraint
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="22"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="30"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -31,6 +31,14 @@
     <sheet name="Talk mutually-exclusive-talks tag 3" sheetId="21" state="visible" r:id="rId22"/>
     <sheet name="Talk mutually-exclusive-talks tag 4" sheetId="22" state="visible" r:id="rId23"/>
     <sheet name="Talk mutually-exclusive-talks tag 5" sheetId="23" state="visible" r:id="rId24"/>
+    <sheet name="Talk prerequisite talks" sheetId="24" state="visible" r:id="rId25"/>
+    <sheet name="Talk prerequisite talks 2" sheetId="25" state="visible" r:id="rId26"/>
+    <sheet name="Talk prerequisite talks 3" sheetId="26" state="visible" r:id="rId27"/>
+    <sheet name="Talk prerequisite talks 4" sheetId="27" state="visible" r:id="rId28"/>
+    <sheet name="Talk prerequisite talks 5" sheetId="28" state="visible" r:id="rId29"/>
+    <sheet name="Talk prerequisite talks 6" sheetId="29" state="visible" r:id="rId30"/>
+    <sheet name="Talk prerequisite talks 7" sheetId="30" state="visible" r:id="rId31"/>
+    <sheet name="Talk prerequisite talks 8" sheetId="31" state="visible" r:id="rId32"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -42,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="153">
   <si>
     <t xml:space="preserve">Conference name</t>
   </si>
@@ -266,6 +274,9 @@
     <t xml:space="preserve">11:00</t>
   </si>
   <si>
+    <t xml:space="preserve">12:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">Name</t>
   </si>
   <si>
@@ -407,6 +418,43 @@
     <t xml:space="preserve">RedHat talk 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Talk with Normal talk as prerequisite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Talk with Normal talk and Normal talk 2 as prerequisites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normal talk, Normal talk2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Talk with (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Talk with Normal talk as prerequisite</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) as a prerequisite</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Constraint package</t>
   </si>
   <si>
@@ -477,6 +525,15 @@
   </si>
   <si>
     <t xml:space="preserve">-3hard/0soft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Talk scheduled after its prerequisites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:00-12:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Talk scheduled before its prerequisites</t>
   </si>
 </sst>
 </file>
@@ -487,7 +544,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -515,6 +572,11 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -634,7 +696,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -658,11 +720,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1158,10 +1220,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1176,7 +1238,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>39</v>
@@ -1197,7 +1259,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1212,10 +1274,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1262,16 +1324,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -1285,14 +1347,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -1344,10 +1406,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1362,7 +1424,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>39</v>
@@ -1383,7 +1445,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1398,10 +1460,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1448,16 +1510,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -1471,13 +1533,13 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -1529,10 +1591,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1547,7 +1609,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>39</v>
@@ -1568,7 +1630,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1583,10 +1645,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1633,16 +1695,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -1656,10 +1718,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -1673,11 +1735,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -1729,10 +1791,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1747,7 +1809,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -1768,7 +1830,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1783,10 +1845,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1833,16 +1895,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -1856,10 +1918,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -1912,10 +1974,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1930,7 +1992,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -1951,7 +2013,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1966,10 +2028,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2016,16 +2078,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -2039,11 +2101,11 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -2096,10 +2158,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2114,7 +2176,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -2135,7 +2197,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2150,10 +2212,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2200,16 +2262,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -2223,10 +2285,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -2279,10 +2341,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2297,7 +2359,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -2318,7 +2380,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2333,10 +2395,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2383,16 +2445,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -2406,10 +2468,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -2462,10 +2524,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2480,7 +2542,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -2501,7 +2563,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2516,10 +2578,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2566,16 +2628,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -2589,14 +2651,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -2648,10 +2710,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2666,7 +2728,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>43</v>
@@ -2687,7 +2749,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2702,10 +2764,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2752,16 +2814,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -2775,10 +2837,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -2792,11 +2854,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -2848,10 +2910,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2866,7 +2928,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -2887,7 +2949,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2902,10 +2964,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2952,16 +3014,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -2975,13 +3037,13 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -3093,7 +3155,20 @@
       </c>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3137,10 +3212,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3155,7 +3230,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3176,7 +3251,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3191,10 +3266,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3241,16 +3316,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -3264,10 +3339,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D8" s="20"/>
       <c r="E8" s="15"/>
@@ -3282,10 +3357,10 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
@@ -3338,10 +3413,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3356,7 +3431,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3377,7 +3452,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3392,10 +3467,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3442,16 +3517,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -3465,10 +3540,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -3484,11 +3559,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -3540,10 +3615,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3558,7 +3633,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3579,7 +3654,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3594,10 +3669,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3644,16 +3719,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -3667,14 +3742,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -3688,11 +3763,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -3744,10 +3819,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3762,7 +3837,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3783,7 +3858,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3798,10 +3873,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3848,16 +3923,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -3871,10 +3946,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -3890,11 +3965,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -3909,12 +3984,1162 @@
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>120</v>
-      </c>
-    </row>
+      <c r="B9" s="15"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+    </row>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+    </row>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="17.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="5" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:E6"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3965,7 +5190,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>64</v>
@@ -3974,18 +5199,18 @@
         <v>65</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>69</v>
@@ -3997,7 +5222,7 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>69</v>
@@ -4009,7 +5234,7 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>69</v>
@@ -4021,7 +5246,7 @@
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>69</v>
@@ -4034,6 +5259,378 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D1:F1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF00DCFF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="26.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="3" style="8" width="19.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="27" style="8" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -4088,40 +5685,40 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
@@ -4129,7 +5726,7 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -4148,7 +5745,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -4167,7 +5764,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -4186,7 +5783,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4255,70 +5852,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>62</v>
@@ -4327,19 +5924,19 @@
         <v>63</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -4365,14 +5962,14 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -4398,14 +5995,14 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -4431,14 +6028,14 @@
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -4464,14 +6061,14 @@
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -4497,7 +6094,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
@@ -4519,7 +6116,7 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="T7" s="2"/>
       <c r="U7" s="6"/>
@@ -4530,18 +6127,18 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>69</v>
       </c>
       <c r="S8" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
@@ -4563,7 +6160,7 @@
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
       <c r="S9" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="T9" s="2"/>
       <c r="U9" s="6"/>
@@ -4572,10 +6169,14 @@
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -4592,17 +6193,23 @@
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
+      <c r="T10" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="U10" s="6"/>
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -4619,17 +6226,23 @@
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
+      <c r="T11" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="U11" s="6"/>
       <c r="V11" s="2"/>
       <c r="W11" s="2"/>
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
+    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>125</v>
+      </c>
       <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -4646,7 +6259,9 @@
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
-      <c r="T12" s="2"/>
+      <c r="T12" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="U12" s="6"/>
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
@@ -6112,10 +7727,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -6130,7 +7745,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>33</v>
@@ -6151,7 +7766,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -6166,10 +7781,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -6216,16 +7831,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -6239,10 +7854,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="16"/>
@@ -6296,10 +7911,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -6314,7 +7929,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>33</v>
@@ -6335,7 +7950,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -6350,10 +7965,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -6400,16 +8015,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -6423,11 +8038,11 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="3"/>
@@ -6480,10 +8095,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -6498,7 +8113,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>37</v>
@@ -6519,7 +8134,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -6534,10 +8149,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -6584,16 +8199,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -6607,10 +8222,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="16"/>
@@ -6664,10 +8279,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -6682,7 +8297,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>37</v>
@@ -6703,7 +8318,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -6718,10 +8333,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -6768,16 +8383,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -6791,10 +8406,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>

</xml_diff>

<commit_message>
Implement Talk mutually-exclusive-talks tag constraint and fix typos in test file
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="30"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="153">
   <si>
     <t xml:space="preserve">Conference name</t>
   </si>
@@ -289,6 +289,9 @@
     <t xml:space="preserve">10:00-11:00</t>
   </si>
   <si>
+    <t xml:space="preserve">11:00-12:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">Normal room</t>
   </si>
   <si>
@@ -424,7 +427,7 @@
     <t xml:space="preserve">Talk with Normal talk and Normal talk 2 as prerequisites</t>
   </si>
   <si>
-    <t xml:space="preserve">Normal talk, Normal talk2</t>
+    <t xml:space="preserve">Normal talk, Normal talk 2</t>
   </si>
   <si>
     <r>
@@ -528,9 +531,6 @@
   </si>
   <si>
     <t xml:space="preserve">Talk scheduled after its prerequisites</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:00-12:00</t>
   </si>
   <si>
     <t xml:space="preserve">Talk scheduled before its prerequisites</t>
@@ -1220,10 +1220,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1238,7 +1238,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>39</v>
@@ -1259,7 +1259,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1274,10 +1274,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1324,7 +1324,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -1347,14 +1347,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -1406,10 +1406,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>39</v>
@@ -1445,7 +1445,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1460,10 +1460,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1510,7 +1510,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -1533,13 +1533,13 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -1591,10 +1591,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1609,7 +1609,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>39</v>
@@ -1630,7 +1630,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1645,10 +1645,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -1718,10 +1718,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -1735,11 +1735,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -1791,10 +1791,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1809,7 +1809,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -1830,7 +1830,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1845,10 +1845,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1895,7 +1895,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -1918,10 +1918,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -1974,10 +1974,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -1992,7 +1992,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -2013,7 +2013,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2078,7 +2078,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -2101,11 +2101,11 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -2158,10 +2158,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2176,7 +2176,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -2197,7 +2197,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2212,10 +2212,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2262,7 +2262,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -2285,10 +2285,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -2341,10 +2341,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2359,7 +2359,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -2380,7 +2380,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2395,10 +2395,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2445,7 +2445,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -2468,10 +2468,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>
@@ -2524,10 +2524,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2542,7 +2542,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>41</v>
@@ -2563,7 +2563,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2578,10 +2578,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2628,7 +2628,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -2651,14 +2651,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -2710,10 +2710,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2728,7 +2728,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>43</v>
@@ -2749,7 +2749,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2764,10 +2764,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2814,7 +2814,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -2837,10 +2837,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -2854,11 +2854,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -2910,10 +2910,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2928,7 +2928,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -2949,7 +2949,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -2964,10 +2964,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3014,7 +3014,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -3037,13 +3037,13 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -3212,10 +3212,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3251,7 +3251,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3266,10 +3266,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3316,7 +3316,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -3339,10 +3339,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D8" s="20"/>
       <c r="E8" s="15"/>
@@ -3357,10 +3357,10 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
@@ -3413,10 +3413,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3431,7 +3431,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3452,7 +3452,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3467,10 +3467,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3517,7 +3517,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -3540,10 +3540,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -3559,11 +3559,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -3615,10 +3615,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3633,7 +3633,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3654,7 +3654,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3669,10 +3669,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3719,7 +3719,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -3742,14 +3742,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -3763,11 +3763,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -3819,10 +3819,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -3837,7 +3837,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>57</v>
@@ -3858,7 +3858,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -3873,10 +3873,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -3923,7 +3923,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -3946,10 +3946,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -3965,11 +3965,11 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="15"/>
@@ -3984,10 +3984,10 @@
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4028,10 +4028,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -4046,7 +4046,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -4067,7 +4067,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -4082,10 +4082,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -4132,7 +4132,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -4155,14 +4155,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="16" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -4176,7 +4176,7 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="20"/>
@@ -4230,10 +4230,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -4248,7 +4248,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -4269,7 +4269,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -4284,10 +4284,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -4334,7 +4334,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -4357,14 +4357,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -4378,10 +4378,10 @@
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C9" s="20"/>
       <c r="D9" s="16"/>
@@ -4436,10 +4436,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -4454,7 +4454,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -4475,7 +4475,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -4490,10 +4490,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -4540,7 +4540,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -4552,7 +4552,7 @@
         <v>78</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>151</v>
+        <v>79</v>
       </c>
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
@@ -4565,17 +4565,17 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
@@ -4626,10 +4626,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -4644,7 +4644,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -4680,10 +4680,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -4730,7 +4730,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -4753,10 +4753,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -4810,10 +4810,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -4828,7 +4828,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -4864,10 +4864,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -4914,7 +4914,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -4937,10 +4937,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -4994,10 +4994,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -5012,7 +5012,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -5048,10 +5048,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -5098,7 +5098,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -5121,10 +5121,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -5166,15 +5166,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="11.86"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1014" min="7" style="0" width="8.67"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1014" min="8" style="0" width="8.67"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="1015" style="0" width="11.52"/>
   </cols>
   <sheetData>
@@ -5187,8 +5187,9 @@
       </c>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G1" s="4"/>
+    </row>
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>75</v>
       </c>
@@ -5207,10 +5208,13 @@
       <c r="F2" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>69</v>
@@ -5222,7 +5226,7 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>69</v>
@@ -5234,7 +5238,7 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>69</v>
@@ -5246,7 +5250,7 @@
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>69</v>
@@ -5258,7 +5262,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D1:G1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -5287,10 +5291,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -5305,7 +5309,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -5341,10 +5345,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -5391,7 +5395,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -5414,14 +5418,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -5473,10 +5477,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -5491,7 +5495,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>59</v>
@@ -5527,10 +5531,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -5577,7 +5581,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -5600,14 +5604,14 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16"/>
@@ -5688,28 +5692,28 @@
         <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>76</v>
@@ -5720,13 +5724,15 @@
       <c r="L2" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="M2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>79</v>
+      </c>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -5745,7 +5751,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -5764,7 +5770,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -5783,7 +5789,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -5801,9 +5807,8 @@
       <c r="O6" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:O1"/>
+  <mergeCells count="1">
+    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -5852,70 +5857,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>62</v>
@@ -5924,19 +5929,19 @@
         <v>63</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -5962,14 +5967,14 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -5995,14 +6000,14 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -6028,14 +6033,14 @@
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -6061,14 +6066,14 @@
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -6094,7 +6099,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
@@ -6116,7 +6121,7 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="T7" s="2"/>
       <c r="U7" s="6"/>
@@ -6127,18 +6132,18 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>69</v>
       </c>
       <c r="S8" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
@@ -6160,7 +6165,7 @@
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
       <c r="S9" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="T9" s="2"/>
       <c r="U9" s="6"/>
@@ -6171,7 +6176,7 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
@@ -6194,7 +6199,7 @@
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
       <c r="T10" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U10" s="6"/>
       <c r="V10" s="2"/>
@@ -6204,7 +6209,7 @@
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
@@ -6227,7 +6232,7 @@
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="U11" s="6"/>
       <c r="V11" s="2"/>
@@ -6237,7 +6242,7 @@
     </row>
     <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
@@ -6260,7 +6265,7 @@
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
       <c r="T12" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="U12" s="6"/>
       <c r="V12" s="2"/>
@@ -7727,10 +7732,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -7745,7 +7750,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>33</v>
@@ -7766,7 +7771,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -7781,10 +7786,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -7831,7 +7836,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -7854,10 +7859,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="16"/>
@@ -7911,10 +7916,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -7929,7 +7934,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>33</v>
@@ -7950,7 +7955,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -7965,10 +7970,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -8015,7 +8020,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>76</v>
@@ -8038,11 +8043,11 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="3"/>
@@ -8095,10 +8100,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -8113,7 +8118,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>37</v>
@@ -8134,7 +8139,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -8149,10 +8154,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -8199,7 +8204,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -8222,10 +8227,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="16"/>
@@ -8279,10 +8284,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -8297,7 +8302,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>37</v>
@@ -8318,7 +8323,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -8333,10 +8338,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -8383,7 +8388,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>76</v>
@@ -8406,10 +8411,10 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="15"/>

</xml_diff>

<commit_message>
Fix typos in constraint names
</commit_message>
<xml_diff>
--- a/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
+++ b/optaplanner-examples/src/test/resources/org/optaplanner/examples/conferencescheduling/solver/testConferenceSchedulingScoreRules.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="22"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="23"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -28,7 +28,7 @@
     <sheet name="Speaker conflict" sheetId="18" state="visible" r:id="rId19"/>
     <sheet name="Talk mutually-exclusive-talks tags" sheetId="19" state="visible" r:id="rId20"/>
     <sheet name="Talk mutually-exclusive-talks tags 2" sheetId="20" state="visible" r:id="rId21"/>
-    <sheet name="Talk mutually-exclusive-talks tag 3" sheetId="21" state="visible" r:id="rId22"/>
+    <sheet name="Talk mutually-exclusive-talks tags 3" sheetId="21" state="visible" r:id="rId22"/>
     <sheet name="Talk mutually-exclusive-talks tags 4" sheetId="22" state="visible" r:id="rId23"/>
     <sheet name="Talk mutually-exclusive-talks tags 5" sheetId="23" state="visible" r:id="rId24"/>
     <sheet name="Talk prerequisite talks" sheetId="24" state="visible" r:id="rId25"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="198">
   <si>
     <t xml:space="preserve">Conference name</t>
   </si>
@@ -629,12 +629,6 @@
   </si>
   <si>
     <t xml:space="preserve">Speaker has conflicting timeslots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Talk mutually-exclusive-talks tag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s</t>
   </si>
   <si>
     <t xml:space="preserve">Mutually exclusive talks in non-overlapping timeslots</t>
@@ -3328,10 +3322,7 @@
         <v>153</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>170</v>
+        <v>63</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -3349,7 +3340,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -3674,10 +3665,7 @@
         <v>153</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>170</v>
+        <v>63</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -3695,7 +3683,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -3878,10 +3866,7 @@
         <v>153</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>170</v>
+        <v>63</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -3899,7 +3884,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -4083,10 +4068,7 @@
         <v>153</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>170</v>
+        <v>63</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -4104,7 +4086,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -4122,7 +4104,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -4290,10 +4272,7 @@
         <v>153</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>170</v>
+        <v>63</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -4311,7 +4290,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -4329,7 +4308,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -4520,7 +4499,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -4722,7 +4701,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -4928,7 +4907,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -5118,7 +5097,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -5302,7 +5281,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -5320,7 +5299,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -5486,7 +5465,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -5842,7 +5821,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -6028,7 +6007,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -6214,7 +6193,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -6400,7 +6379,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -6590,7 +6569,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -6608,7 +6587,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -6780,7 +6759,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -6798,7 +6777,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -6970,7 +6949,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -6988,7 +6967,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -7160,7 +7139,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -7178,7 +7157,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -7352,7 +7331,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -7370,7 +7349,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -7561,7 +7540,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -7579,7 +7558,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -7958,7 +7937,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -7976,7 +7955,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -8167,7 +8146,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -8185,7 +8164,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -8376,7 +8355,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -8394,7 +8373,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -8590,7 +8569,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -8608,7 +8587,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -8804,7 +8783,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -8822,7 +8801,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -9014,7 +8993,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -9032,7 +9011,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -9228,7 +9207,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -9246,7 +9225,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>

</xml_diff>